<commit_message>
Remove the bit column since in MySQL it is not the same as SQL Server
</commit_message>
<xml_diff>
--- a/tests/SQL/fixtures/data/test_mysql.xlsx
+++ b/tests/SQL/fixtures/data/test_mysql.xlsx
@@ -15,13 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="244">
-  <si>
-    <t>bit</t>
-  </si>
-  <si>
-    <t>bit_nullable</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="242">
   <si>
     <t>tinyint</t>
   </si>
@@ -1086,10 +1080,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:CH11"/>
+  <dimension ref="A1:CF11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:86">
+    <row r="1" spans="1:84">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1342,294 +1336,285 @@
       <c r="CF1" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" t="s">
+    </row>
+    <row r="2" spans="1:84">
+      <c r="A2">
+        <v>126</v>
+      </c>
+      <c r="C2">
+        <v>127</v>
+      </c>
+      <c r="E2">
+        <v>254</v>
+      </c>
+      <c r="G2">
+        <v>255</v>
+      </c>
+      <c r="I2">
+        <v>32766</v>
+      </c>
+      <c r="K2">
+        <v>32767</v>
+      </c>
+      <c r="M2">
+        <v>65534</v>
+      </c>
+      <c r="O2">
+        <v>65535</v>
+      </c>
+      <c r="Q2">
+        <v>8388606</v>
+      </c>
+      <c r="S2">
+        <v>8388607</v>
+      </c>
+      <c r="U2">
+        <v>16777214</v>
+      </c>
+      <c r="W2">
+        <v>16777215</v>
+      </c>
+      <c r="Y2">
+        <v>2147483646</v>
+      </c>
+      <c r="AA2">
+        <v>2147483647</v>
+      </c>
+      <c r="AC2">
+        <v>4294967294</v>
+      </c>
+      <c r="AE2">
+        <v>4294967295</v>
+      </c>
+      <c r="AG2">
+        <v>-2147483650</v>
+      </c>
+      <c r="AI2">
+        <v>-2147483649</v>
+      </c>
+      <c r="AK2">
+        <v>4294967305</v>
+      </c>
+      <c r="AM2">
+        <v>4294967306</v>
+      </c>
+      <c r="AO2">
+        <v>9999999.98000000044703</v>
+      </c>
+      <c r="AQ2">
+        <v>9999999.99000000022352</v>
+      </c>
+      <c r="AS2">
+        <v>99999999.97999998927116</v>
+      </c>
+      <c r="AU2">
+        <v>99999999.98999999463558</v>
+      </c>
+      <c r="AW2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AY2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BA2" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="BC2" t="s">
         <v>85</v>
       </c>
+      <c r="BE2" t="s">
+        <v>86</v>
+      </c>
+      <c r="BG2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>89</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>92</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>93</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>95</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>96</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>97</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>98</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>99</v>
+      </c>
     </row>
-    <row r="2" spans="1:86">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
+    <row r="3" spans="1:84">
+      <c r="A3">
         <v>126</v>
       </c>
-      <c r="E2">
-        <v>127</v>
-      </c>
-      <c r="G2">
-        <v>254</v>
-      </c>
-      <c r="I2">
-        <v>255</v>
-      </c>
-      <c r="K2">
-        <v>32766</v>
-      </c>
-      <c r="M2">
-        <v>32767</v>
-      </c>
-      <c r="O2">
-        <v>65534</v>
-      </c>
-      <c r="Q2">
-        <v>65535</v>
-      </c>
-      <c r="S2">
-        <v>8388606</v>
-      </c>
-      <c r="U2">
-        <v>8388607</v>
-      </c>
-      <c r="W2">
-        <v>16777214</v>
-      </c>
-      <c r="Y2">
-        <v>16777215</v>
-      </c>
-      <c r="AA2">
-        <v>2147483646</v>
-      </c>
-      <c r="AC2">
-        <v>2147483647</v>
-      </c>
-      <c r="AE2">
-        <v>4294967294</v>
-      </c>
-      <c r="AG2">
-        <v>4294967295</v>
-      </c>
-      <c r="AI2">
-        <v>-2147483650</v>
-      </c>
-      <c r="AK2">
-        <v>-2147483649</v>
-      </c>
-      <c r="AM2">
-        <v>4294967305</v>
-      </c>
-      <c r="AO2">
-        <v>4294967306</v>
-      </c>
-      <c r="AQ2">
-        <v>9999999.98000000044703</v>
-      </c>
-      <c r="AS2">
-        <v>9999999.99000000022352</v>
-      </c>
-      <c r="AU2">
-        <v>99999999.97999998927116</v>
-      </c>
-      <c r="AW2">
-        <v>99999999.98999999463558</v>
-      </c>
-      <c r="AY2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BA2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>86</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>87</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>89</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>90</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>92</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>93</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>95</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>96</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>97</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>98</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>99</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>100</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:86">
-      <c r="A3">
-        <v>0</v>
+      <c r="B3">
+        <v>125</v>
       </c>
       <c r="C3">
         <v>126</v>
       </c>
       <c r="D3">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E3">
-        <v>126</v>
+        <v>254</v>
       </c>
       <c r="F3">
-        <v>126</v>
+        <v>253</v>
       </c>
       <c r="G3">
         <v>254</v>
       </c>
       <c r="H3">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I3">
-        <v>254</v>
+        <v>32766</v>
       </c>
       <c r="J3">
-        <v>254</v>
+        <v>32765</v>
       </c>
       <c r="K3">
         <v>32766</v>
       </c>
       <c r="L3">
-        <v>32765</v>
+        <v>32766</v>
       </c>
       <c r="M3">
-        <v>32766</v>
+        <v>65534</v>
       </c>
       <c r="N3">
-        <v>32766</v>
+        <v>65533</v>
       </c>
       <c r="O3">
         <v>65534</v>
       </c>
       <c r="P3">
-        <v>65533</v>
+        <v>65534</v>
       </c>
       <c r="Q3">
-        <v>65534</v>
+        <v>8388606</v>
       </c>
       <c r="R3">
-        <v>65534</v>
+        <v>8388605</v>
       </c>
       <c r="S3">
         <v>8388606</v>
       </c>
       <c r="T3">
-        <v>8388605</v>
+        <v>8388606</v>
       </c>
       <c r="U3">
-        <v>8388606</v>
+        <v>16777214</v>
       </c>
       <c r="V3">
-        <v>8388606</v>
+        <v>16777213</v>
       </c>
       <c r="W3">
         <v>16777214</v>
       </c>
       <c r="X3">
-        <v>16777213</v>
+        <v>16777214</v>
       </c>
       <c r="Y3">
-        <v>16777214</v>
+        <v>2147483646</v>
       </c>
       <c r="Z3">
-        <v>16777214</v>
+        <v>2147483645</v>
       </c>
       <c r="AA3">
         <v>2147483646</v>
       </c>
       <c r="AB3">
-        <v>2147483645</v>
+        <v>2147483646</v>
       </c>
       <c r="AC3">
-        <v>2147483646</v>
+        <v>4294967294</v>
       </c>
       <c r="AD3">
-        <v>2147483646</v>
+        <v>4294967293</v>
       </c>
       <c r="AE3">
         <v>4294967294</v>
       </c>
       <c r="AF3">
-        <v>4294967293</v>
+        <v>4294967294</v>
       </c>
       <c r="AG3">
-        <v>4294967294</v>
+        <v>-2147483650</v>
       </c>
       <c r="AH3">
-        <v>4294967294</v>
+        <v>-2147483651</v>
       </c>
       <c r="AI3">
         <v>-2147483650</v>
       </c>
       <c r="AJ3">
-        <v>-2147483651</v>
+        <v>-2147483650</v>
       </c>
       <c r="AK3">
-        <v>-2147483650</v>
+        <v>4294967305</v>
       </c>
       <c r="AL3">
-        <v>-2147483650</v>
+        <v>4294967304</v>
       </c>
       <c r="AM3">
         <v>4294967305</v>
       </c>
       <c r="AN3">
-        <v>4294967304</v>
+        <v>4294967305</v>
       </c>
       <c r="AO3">
-        <v>4294967305</v>
+        <v>9999999.98000000044703</v>
       </c>
       <c r="AP3">
-        <v>4294967305</v>
+        <v>9999999.97000000067055</v>
       </c>
       <c r="AQ3">
         <v>9999999.98000000044703</v>
       </c>
       <c r="AR3">
-        <v>9999999.97000000067055</v>
+        <v>9999999.98000000044703</v>
       </c>
       <c r="AS3">
-        <v>9999999.98000000044703</v>
+        <v>99999999.97999998927116</v>
       </c>
       <c r="AT3">
-        <v>9999999.98000000044703</v>
+        <v>99999999.96999999880791</v>
       </c>
       <c r="AU3">
         <v>99999999.97999998927116</v>
       </c>
       <c r="AV3">
-        <v>99999999.96999999880791</v>
-      </c>
-      <c r="AW3">
         <v>99999999.97999998927116</v>
       </c>
-      <c r="AX3">
-        <v>99999999.97999998927116</v>
+      <c r="AW3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX3" t="b">
+        <v>1</v>
       </c>
       <c r="AY3" t="b">
         <v>1</v>
@@ -1637,115 +1622,109 @@
       <c r="AZ3" t="b">
         <v>1</v>
       </c>
-      <c r="BA3" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB3" t="b">
-        <v>1</v>
+      <c r="BA3" t="s">
+        <v>84</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>100</v>
       </c>
       <c r="BC3" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="BD3" t="s">
         <v>102</v>
       </c>
       <c r="BE3" t="s">
+        <v>86</v>
+      </c>
+      <c r="BF3" t="s">
         <v>103</v>
       </c>
-      <c r="BF3" t="s">
+      <c r="BG3" t="s">
         <v>104</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>88</v>
       </c>
       <c r="BH3" t="s">
         <v>105</v>
       </c>
       <c r="BI3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BJ3" t="s">
         <v>106</v>
       </c>
-      <c r="BJ3" t="s">
+      <c r="BK3" t="s">
         <v>107</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>90</v>
       </c>
       <c r="BL3" t="s">
         <v>108</v>
       </c>
       <c r="BM3" t="s">
+        <v>90</v>
+      </c>
+      <c r="BN3" t="s">
         <v>109</v>
       </c>
-      <c r="BN3" t="s">
-        <v>110</v>
-      </c>
       <c r="BO3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="BP3" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="BQ3" t="s">
         <v>92</v>
       </c>
       <c r="BR3" t="s">
+        <v>110</v>
+      </c>
+      <c r="BS3" t="s">
         <v>92</v>
       </c>
-      <c r="BS3" t="s">
-        <v>94</v>
-      </c>
       <c r="BT3" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="BU3" t="s">
         <v>94</v>
       </c>
       <c r="BV3" t="s">
+        <v>111</v>
+      </c>
+      <c r="BW3" t="s">
         <v>94</v>
       </c>
-      <c r="BW3" t="s">
-        <v>96</v>
-      </c>
       <c r="BX3" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="BY3" t="s">
         <v>96</v>
       </c>
       <c r="BZ3" t="s">
+        <v>112</v>
+      </c>
+      <c r="CA3" t="s">
         <v>96</v>
       </c>
-      <c r="CA3" t="s">
-        <v>98</v>
-      </c>
       <c r="CB3" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="CC3" t="s">
         <v>98</v>
       </c>
       <c r="CD3" t="s">
+        <v>113</v>
+      </c>
+      <c r="CE3" t="s">
         <v>98</v>
       </c>
-      <c r="CE3" t="s">
-        <v>100</v>
-      </c>
       <c r="CF3" t="s">
-        <v>115</v>
-      </c>
-      <c r="CG3" t="s">
-        <v>100</v>
-      </c>
-      <c r="CH3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:86">
+    <row r="4" spans="1:84">
       <c r="A4">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="C4">
         <v>125</v>
@@ -1754,10 +1733,10 @@
         <v>125</v>
       </c>
       <c r="E4">
-        <v>125</v>
+        <v>253</v>
       </c>
       <c r="F4">
-        <v>125</v>
+        <v>253</v>
       </c>
       <c r="G4">
         <v>253</v>
@@ -1766,10 +1745,10 @@
         <v>253</v>
       </c>
       <c r="I4">
-        <v>253</v>
+        <v>32765</v>
       </c>
       <c r="J4">
-        <v>253</v>
+        <v>32765</v>
       </c>
       <c r="K4">
         <v>32765</v>
@@ -1778,10 +1757,10 @@
         <v>32765</v>
       </c>
       <c r="M4">
-        <v>32765</v>
+        <v>65533</v>
       </c>
       <c r="N4">
-        <v>32765</v>
+        <v>65533</v>
       </c>
       <c r="O4">
         <v>65533</v>
@@ -1790,10 +1769,10 @@
         <v>65533</v>
       </c>
       <c r="Q4">
-        <v>65533</v>
+        <v>8388605</v>
       </c>
       <c r="R4">
-        <v>65533</v>
+        <v>8388605</v>
       </c>
       <c r="S4">
         <v>8388605</v>
@@ -1802,10 +1781,10 @@
         <v>8388605</v>
       </c>
       <c r="U4">
-        <v>8388605</v>
+        <v>16777213</v>
       </c>
       <c r="V4">
-        <v>8388605</v>
+        <v>16777213</v>
       </c>
       <c r="W4">
         <v>16777213</v>
@@ -1814,10 +1793,10 @@
         <v>16777213</v>
       </c>
       <c r="Y4">
-        <v>16777213</v>
+        <v>2147483645</v>
       </c>
       <c r="Z4">
-        <v>16777213</v>
+        <v>2147483645</v>
       </c>
       <c r="AA4">
         <v>2147483645</v>
@@ -1826,10 +1805,10 @@
         <v>2147483645</v>
       </c>
       <c r="AC4">
-        <v>2147483645</v>
+        <v>4294967293</v>
       </c>
       <c r="AD4">
-        <v>2147483645</v>
+        <v>4294967293</v>
       </c>
       <c r="AE4">
         <v>4294967293</v>
@@ -1838,10 +1817,10 @@
         <v>4294967293</v>
       </c>
       <c r="AG4">
-        <v>4294967293</v>
+        <v>-2147483651</v>
       </c>
       <c r="AH4">
-        <v>4294967293</v>
+        <v>-2147483651</v>
       </c>
       <c r="AI4">
         <v>-2147483651</v>
@@ -1850,10 +1829,10 @@
         <v>-2147483651</v>
       </c>
       <c r="AK4">
-        <v>-2147483651</v>
+        <v>4294967304</v>
       </c>
       <c r="AL4">
-        <v>-2147483651</v>
+        <v>4294967304</v>
       </c>
       <c r="AM4">
         <v>4294967304</v>
@@ -1862,10 +1841,10 @@
         <v>4294967304</v>
       </c>
       <c r="AO4">
-        <v>4294967304</v>
+        <v>9999999.97000000067055</v>
       </c>
       <c r="AP4">
-        <v>4294967304</v>
+        <v>9999999.97000000067055</v>
       </c>
       <c r="AQ4">
         <v>9999999.97000000067055</v>
@@ -1874,10 +1853,10 @@
         <v>9999999.97000000067055</v>
       </c>
       <c r="AS4">
-        <v>9999999.97000000067055</v>
+        <v>99999999.96999999880791</v>
       </c>
       <c r="AT4">
-        <v>9999999.97000000067055</v>
+        <v>99999999.96999999880791</v>
       </c>
       <c r="AU4">
         <v>99999999.96999999880791</v>
@@ -1885,11 +1864,11 @@
       <c r="AV4">
         <v>99999999.96999999880791</v>
       </c>
-      <c r="AW4">
-        <v>99999999.96999999880791</v>
-      </c>
-      <c r="AX4">
-        <v>99999999.96999999880791</v>
+      <c r="AW4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX4" t="b">
+        <v>1</v>
       </c>
       <c r="AY4" t="b">
         <v>1</v>
@@ -1897,115 +1876,109 @@
       <c r="AZ4" t="b">
         <v>1</v>
       </c>
-      <c r="BA4" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB4" t="b">
-        <v>1</v>
+      <c r="BA4" t="s">
+        <v>114</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>100</v>
       </c>
       <c r="BC4" t="s">
+        <v>115</v>
+      </c>
+      <c r="BD4" t="s">
         <v>116</v>
-      </c>
-      <c r="BD4" t="s">
-        <v>102</v>
       </c>
       <c r="BE4" t="s">
         <v>117</v>
       </c>
       <c r="BF4" t="s">
+        <v>103</v>
+      </c>
+      <c r="BG4" t="s">
         <v>118</v>
       </c>
-      <c r="BG4" t="s">
+      <c r="BH4" t="s">
         <v>119</v>
-      </c>
-      <c r="BH4" t="s">
-        <v>105</v>
       </c>
       <c r="BI4" t="s">
         <v>120</v>
       </c>
       <c r="BJ4" t="s">
+        <v>106</v>
+      </c>
+      <c r="BK4" t="s">
         <v>121</v>
       </c>
-      <c r="BK4" t="s">
+      <c r="BL4" t="s">
         <v>122</v>
       </c>
-      <c r="BL4" t="s">
-        <v>108</v>
-      </c>
       <c r="BM4" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="BN4" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>109</v>
+      </c>
+      <c r="BP4" t="s">
+        <v>109</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>110</v>
+      </c>
+      <c r="BR4" t="s">
+        <v>110</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>110</v>
+      </c>
+      <c r="BT4" t="s">
+        <v>110</v>
+      </c>
+      <c r="BU4" t="s">
+        <v>111</v>
+      </c>
+      <c r="BV4" t="s">
+        <v>111</v>
+      </c>
+      <c r="BW4" t="s">
+        <v>111</v>
+      </c>
+      <c r="BX4" t="s">
+        <v>111</v>
+      </c>
+      <c r="BY4" t="s">
+        <v>112</v>
+      </c>
+      <c r="BZ4" t="s">
+        <v>112</v>
+      </c>
+      <c r="CA4" t="s">
+        <v>112</v>
+      </c>
+      <c r="CB4" t="s">
+        <v>112</v>
+      </c>
+      <c r="CC4" t="s">
+        <v>113</v>
+      </c>
+      <c r="CD4" t="s">
+        <v>113</v>
+      </c>
+      <c r="CE4" t="s">
+        <v>113</v>
+      </c>
+      <c r="CF4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:84">
+      <c r="A5">
         <v>124</v>
       </c>
-      <c r="BO4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BP4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BQ4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BR4" t="s">
-        <v>111</v>
-      </c>
-      <c r="BS4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BT4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BU4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BV4" t="s">
-        <v>112</v>
-      </c>
-      <c r="BW4" t="s">
-        <v>113</v>
-      </c>
-      <c r="BX4" t="s">
-        <v>113</v>
-      </c>
-      <c r="BY4" t="s">
-        <v>113</v>
-      </c>
-      <c r="BZ4" t="s">
-        <v>113</v>
-      </c>
-      <c r="CA4" t="s">
-        <v>114</v>
-      </c>
-      <c r="CB4" t="s">
-        <v>114</v>
-      </c>
-      <c r="CC4" t="s">
-        <v>114</v>
-      </c>
-      <c r="CD4" t="s">
-        <v>114</v>
-      </c>
-      <c r="CE4" t="s">
-        <v>115</v>
-      </c>
-      <c r="CF4" t="s">
-        <v>115</v>
-      </c>
-      <c r="CG4" t="s">
-        <v>115</v>
-      </c>
-      <c r="CH4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:86">
-      <c r="A5">
-        <v>0</v>
-      </c>
       <c r="B5">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="C5">
         <v>124</v>
@@ -2014,10 +1987,10 @@
         <v>124</v>
       </c>
       <c r="E5">
-        <v>124</v>
+        <v>252</v>
       </c>
       <c r="F5">
-        <v>124</v>
+        <v>252</v>
       </c>
       <c r="G5">
         <v>252</v>
@@ -2026,10 +1999,10 @@
         <v>252</v>
       </c>
       <c r="I5">
-        <v>252</v>
+        <v>32764</v>
       </c>
       <c r="J5">
-        <v>252</v>
+        <v>32764</v>
       </c>
       <c r="K5">
         <v>32764</v>
@@ -2038,10 +2011,10 @@
         <v>32764</v>
       </c>
       <c r="M5">
-        <v>32764</v>
+        <v>65532</v>
       </c>
       <c r="N5">
-        <v>32764</v>
+        <v>65532</v>
       </c>
       <c r="O5">
         <v>65532</v>
@@ -2050,10 +2023,10 @@
         <v>65532</v>
       </c>
       <c r="Q5">
-        <v>65532</v>
+        <v>8388604</v>
       </c>
       <c r="R5">
-        <v>65532</v>
+        <v>8388604</v>
       </c>
       <c r="S5">
         <v>8388604</v>
@@ -2062,10 +2035,10 @@
         <v>8388604</v>
       </c>
       <c r="U5">
-        <v>8388604</v>
+        <v>16777212</v>
       </c>
       <c r="V5">
-        <v>8388604</v>
+        <v>16777212</v>
       </c>
       <c r="W5">
         <v>16777212</v>
@@ -2074,10 +2047,10 @@
         <v>16777212</v>
       </c>
       <c r="Y5">
-        <v>16777212</v>
+        <v>2147483644</v>
       </c>
       <c r="Z5">
-        <v>16777212</v>
+        <v>2147483644</v>
       </c>
       <c r="AA5">
         <v>2147483644</v>
@@ -2086,10 +2059,10 @@
         <v>2147483644</v>
       </c>
       <c r="AC5">
-        <v>2147483644</v>
+        <v>4294967292</v>
       </c>
       <c r="AD5">
-        <v>2147483644</v>
+        <v>4294967292</v>
       </c>
       <c r="AE5">
         <v>4294967292</v>
@@ -2098,10 +2071,10 @@
         <v>4294967292</v>
       </c>
       <c r="AG5">
-        <v>4294967292</v>
+        <v>-2147483652</v>
       </c>
       <c r="AH5">
-        <v>4294967292</v>
+        <v>-2147483652</v>
       </c>
       <c r="AI5">
         <v>-2147483652</v>
@@ -2110,10 +2083,10 @@
         <v>-2147483652</v>
       </c>
       <c r="AK5">
-        <v>-2147483652</v>
+        <v>4294967303</v>
       </c>
       <c r="AL5">
-        <v>-2147483652</v>
+        <v>4294967303</v>
       </c>
       <c r="AM5">
         <v>4294967303</v>
@@ -2122,10 +2095,10 @@
         <v>4294967303</v>
       </c>
       <c r="AO5">
-        <v>4294967303</v>
+        <v>9999999.96000000089407</v>
       </c>
       <c r="AP5">
-        <v>4294967303</v>
+        <v>9999999.96000000089407</v>
       </c>
       <c r="AQ5">
         <v>9999999.96000000089407</v>
@@ -2134,10 +2107,10 @@
         <v>9999999.96000000089407</v>
       </c>
       <c r="AS5">
-        <v>9999999.96000000089407</v>
+        <v>99999999.95999999344349</v>
       </c>
       <c r="AT5">
-        <v>9999999.96000000089407</v>
+        <v>99999999.95999999344349</v>
       </c>
       <c r="AU5">
         <v>99999999.95999999344349</v>
@@ -2145,11 +2118,11 @@
       <c r="AV5">
         <v>99999999.95999999344349</v>
       </c>
-      <c r="AW5">
-        <v>99999999.95999999344349</v>
-      </c>
-      <c r="AX5">
-        <v>99999999.95999999344349</v>
+      <c r="AW5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX5" t="b">
+        <v>1</v>
       </c>
       <c r="AY5" t="b">
         <v>1</v>
@@ -2157,11 +2130,11 @@
       <c r="AZ5" t="b">
         <v>1</v>
       </c>
-      <c r="BA5" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB5" t="b">
-        <v>1</v>
+      <c r="BA5" t="s">
+        <v>123</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>124</v>
       </c>
       <c r="BC5" t="s">
         <v>125</v>
@@ -2197,75 +2170,69 @@
         <v>135</v>
       </c>
       <c r="BN5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BO5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BP5" t="s">
+        <v>135</v>
+      </c>
+      <c r="BQ5" t="s">
         <v>136</v>
       </c>
-      <c r="BO5" t="s">
+      <c r="BR5" t="s">
+        <v>136</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>136</v>
+      </c>
+      <c r="BT5" t="s">
+        <v>136</v>
+      </c>
+      <c r="BU5" t="s">
         <v>137</v>
       </c>
-      <c r="BP5" t="s">
+      <c r="BV5" t="s">
         <v>137</v>
       </c>
-      <c r="BQ5" t="s">
+      <c r="BW5" t="s">
         <v>137</v>
       </c>
-      <c r="BR5" t="s">
+      <c r="BX5" t="s">
         <v>137</v>
       </c>
-      <c r="BS5" t="s">
+      <c r="BY5" t="s">
         <v>138</v>
       </c>
-      <c r="BT5" t="s">
+      <c r="BZ5" t="s">
         <v>138</v>
       </c>
-      <c r="BU5" t="s">
+      <c r="CA5" t="s">
         <v>138</v>
       </c>
-      <c r="BV5" t="s">
+      <c r="CB5" t="s">
         <v>138</v>
       </c>
-      <c r="BW5" t="s">
+      <c r="CC5" t="s">
         <v>139</v>
       </c>
-      <c r="BX5" t="s">
+      <c r="CD5" t="s">
         <v>139</v>
       </c>
-      <c r="BY5" t="s">
+      <c r="CE5" t="s">
         <v>139</v>
       </c>
-      <c r="BZ5" t="s">
+      <c r="CF5" t="s">
         <v>139</v>
       </c>
-      <c r="CA5" t="s">
-        <v>140</v>
-      </c>
-      <c r="CB5" t="s">
-        <v>140</v>
-      </c>
-      <c r="CC5" t="s">
-        <v>140</v>
-      </c>
-      <c r="CD5" t="s">
-        <v>140</v>
-      </c>
-      <c r="CE5" t="s">
-        <v>141</v>
-      </c>
-      <c r="CF5" t="s">
-        <v>141</v>
-      </c>
-      <c r="CG5" t="s">
-        <v>141</v>
-      </c>
-      <c r="CH5" t="s">
-        <v>141</v>
-      </c>
     </row>
-    <row r="6" spans="1:86">
+    <row r="6" spans="1:84">
       <c r="A6">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -2274,10 +2241,10 @@
         <v>123</v>
       </c>
       <c r="E6">
-        <v>123</v>
+        <v>251</v>
       </c>
       <c r="F6">
-        <v>123</v>
+        <v>251</v>
       </c>
       <c r="G6">
         <v>251</v>
@@ -2286,10 +2253,10 @@
         <v>251</v>
       </c>
       <c r="I6">
-        <v>251</v>
+        <v>32763</v>
       </c>
       <c r="J6">
-        <v>251</v>
+        <v>32763</v>
       </c>
       <c r="K6">
         <v>32763</v>
@@ -2298,10 +2265,10 @@
         <v>32763</v>
       </c>
       <c r="M6">
-        <v>32763</v>
+        <v>65531</v>
       </c>
       <c r="N6">
-        <v>32763</v>
+        <v>65531</v>
       </c>
       <c r="O6">
         <v>65531</v>
@@ -2310,10 +2277,10 @@
         <v>65531</v>
       </c>
       <c r="Q6">
-        <v>65531</v>
+        <v>8388603</v>
       </c>
       <c r="R6">
-        <v>65531</v>
+        <v>8388603</v>
       </c>
       <c r="S6">
         <v>8388603</v>
@@ -2322,10 +2289,10 @@
         <v>8388603</v>
       </c>
       <c r="U6">
-        <v>8388603</v>
+        <v>16777211</v>
       </c>
       <c r="V6">
-        <v>8388603</v>
+        <v>16777211</v>
       </c>
       <c r="W6">
         <v>16777211</v>
@@ -2334,10 +2301,10 @@
         <v>16777211</v>
       </c>
       <c r="Y6">
-        <v>16777211</v>
+        <v>2147483643</v>
       </c>
       <c r="Z6">
-        <v>16777211</v>
+        <v>2147483643</v>
       </c>
       <c r="AA6">
         <v>2147483643</v>
@@ -2346,10 +2313,10 @@
         <v>2147483643</v>
       </c>
       <c r="AC6">
-        <v>2147483643</v>
+        <v>4294967291</v>
       </c>
       <c r="AD6">
-        <v>2147483643</v>
+        <v>4294967291</v>
       </c>
       <c r="AE6">
         <v>4294967291</v>
@@ -2358,10 +2325,10 @@
         <v>4294967291</v>
       </c>
       <c r="AG6">
-        <v>4294967291</v>
+        <v>-2147483653</v>
       </c>
       <c r="AH6">
-        <v>4294967291</v>
+        <v>-2147483653</v>
       </c>
       <c r="AI6">
         <v>-2147483653</v>
@@ -2370,10 +2337,10 @@
         <v>-2147483653</v>
       </c>
       <c r="AK6">
-        <v>-2147483653</v>
+        <v>4294967302</v>
       </c>
       <c r="AL6">
-        <v>-2147483653</v>
+        <v>4294967302</v>
       </c>
       <c r="AM6">
         <v>4294967302</v>
@@ -2382,10 +2349,10 @@
         <v>4294967302</v>
       </c>
       <c r="AO6">
-        <v>4294967302</v>
+        <v>9999999.95000000111759</v>
       </c>
       <c r="AP6">
-        <v>4294967302</v>
+        <v>9999999.95000000111759</v>
       </c>
       <c r="AQ6">
         <v>9999999.95000000111759</v>
@@ -2394,10 +2361,10 @@
         <v>9999999.95000000111759</v>
       </c>
       <c r="AS6">
-        <v>9999999.95000000111759</v>
+        <v>99999999.94999998807907</v>
       </c>
       <c r="AT6">
-        <v>9999999.95000000111759</v>
+        <v>99999999.94999998807907</v>
       </c>
       <c r="AU6">
         <v>99999999.94999998807907</v>
@@ -2405,11 +2372,11 @@
       <c r="AV6">
         <v>99999999.94999998807907</v>
       </c>
-      <c r="AW6">
-        <v>99999999.94999998807907</v>
-      </c>
-      <c r="AX6">
-        <v>99999999.94999998807907</v>
+      <c r="AW6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX6" t="b">
+        <v>1</v>
       </c>
       <c r="AY6" t="b">
         <v>1</v>
@@ -2417,11 +2384,11 @@
       <c r="AZ6" t="b">
         <v>1</v>
       </c>
-      <c r="BA6" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB6" t="b">
-        <v>1</v>
+      <c r="BA6" t="s">
+        <v>140</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>141</v>
       </c>
       <c r="BC6" t="s">
         <v>142</v>
@@ -2457,75 +2424,69 @@
         <v>152</v>
       </c>
       <c r="BN6" t="s">
+        <v>152</v>
+      </c>
+      <c r="BO6" t="s">
+        <v>152</v>
+      </c>
+      <c r="BP6" t="s">
+        <v>152</v>
+      </c>
+      <c r="BQ6" t="s">
         <v>153</v>
       </c>
-      <c r="BO6" t="s">
+      <c r="BR6" t="s">
+        <v>153</v>
+      </c>
+      <c r="BS6" t="s">
+        <v>153</v>
+      </c>
+      <c r="BT6" t="s">
+        <v>153</v>
+      </c>
+      <c r="BU6" t="s">
         <v>154</v>
       </c>
-      <c r="BP6" t="s">
+      <c r="BV6" t="s">
         <v>154</v>
       </c>
-      <c r="BQ6" t="s">
+      <c r="BW6" t="s">
         <v>154</v>
       </c>
-      <c r="BR6" t="s">
+      <c r="BX6" t="s">
         <v>154</v>
       </c>
-      <c r="BS6" t="s">
+      <c r="BY6" t="s">
         <v>155</v>
       </c>
-      <c r="BT6" t="s">
+      <c r="BZ6" t="s">
         <v>155</v>
       </c>
-      <c r="BU6" t="s">
+      <c r="CA6" t="s">
         <v>155</v>
       </c>
-      <c r="BV6" t="s">
+      <c r="CB6" t="s">
         <v>155</v>
       </c>
-      <c r="BW6" t="s">
+      <c r="CC6" t="s">
         <v>156</v>
       </c>
-      <c r="BX6" t="s">
+      <c r="CD6" t="s">
         <v>156</v>
       </c>
-      <c r="BY6" t="s">
+      <c r="CE6" t="s">
         <v>156</v>
       </c>
-      <c r="BZ6" t="s">
+      <c r="CF6" t="s">
         <v>156</v>
       </c>
-      <c r="CA6" t="s">
-        <v>157</v>
-      </c>
-      <c r="CB6" t="s">
-        <v>157</v>
-      </c>
-      <c r="CC6" t="s">
-        <v>157</v>
-      </c>
-      <c r="CD6" t="s">
-        <v>157</v>
-      </c>
-      <c r="CE6" t="s">
-        <v>158</v>
-      </c>
-      <c r="CF6" t="s">
-        <v>158</v>
-      </c>
-      <c r="CG6" t="s">
-        <v>158</v>
-      </c>
-      <c r="CH6" t="s">
-        <v>158</v>
-      </c>
     </row>
-    <row r="7" spans="1:86">
+    <row r="7" spans="1:84">
       <c r="A7">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="C7">
         <v>122</v>
@@ -2534,10 +2495,10 @@
         <v>122</v>
       </c>
       <c r="E7">
-        <v>122</v>
+        <v>250</v>
       </c>
       <c r="F7">
-        <v>122</v>
+        <v>250</v>
       </c>
       <c r="G7">
         <v>250</v>
@@ -2546,10 +2507,10 @@
         <v>250</v>
       </c>
       <c r="I7">
-        <v>250</v>
+        <v>32762</v>
       </c>
       <c r="J7">
-        <v>250</v>
+        <v>32762</v>
       </c>
       <c r="K7">
         <v>32762</v>
@@ -2558,10 +2519,10 @@
         <v>32762</v>
       </c>
       <c r="M7">
-        <v>32762</v>
+        <v>65530</v>
       </c>
       <c r="N7">
-        <v>32762</v>
+        <v>65530</v>
       </c>
       <c r="O7">
         <v>65530</v>
@@ -2570,10 +2531,10 @@
         <v>65530</v>
       </c>
       <c r="Q7">
-        <v>65530</v>
+        <v>8388602</v>
       </c>
       <c r="R7">
-        <v>65530</v>
+        <v>8388602</v>
       </c>
       <c r="S7">
         <v>8388602</v>
@@ -2582,10 +2543,10 @@
         <v>8388602</v>
       </c>
       <c r="U7">
-        <v>8388602</v>
+        <v>16777210</v>
       </c>
       <c r="V7">
-        <v>8388602</v>
+        <v>16777210</v>
       </c>
       <c r="W7">
         <v>16777210</v>
@@ -2594,10 +2555,10 @@
         <v>16777210</v>
       </c>
       <c r="Y7">
-        <v>16777210</v>
+        <v>2147483642</v>
       </c>
       <c r="Z7">
-        <v>16777210</v>
+        <v>2147483642</v>
       </c>
       <c r="AA7">
         <v>2147483642</v>
@@ -2606,10 +2567,10 @@
         <v>2147483642</v>
       </c>
       <c r="AC7">
-        <v>2147483642</v>
+        <v>4294967290</v>
       </c>
       <c r="AD7">
-        <v>2147483642</v>
+        <v>4294967290</v>
       </c>
       <c r="AE7">
         <v>4294967290</v>
@@ -2618,16 +2579,16 @@
         <v>4294967290</v>
       </c>
       <c r="AG7">
-        <v>4294967290</v>
-      </c>
-      <c r="AH7">
-        <v>4294967290</v>
+        <v>2147483652</v>
       </c>
       <c r="AI7">
-        <v>2147483652</v>
+        <v>2147483653</v>
       </c>
       <c r="AK7">
-        <v>2147483653</v>
+        <v>4294967301</v>
+      </c>
+      <c r="AL7">
+        <v>4294967301</v>
       </c>
       <c r="AM7">
         <v>4294967301</v>
@@ -2636,10 +2597,10 @@
         <v>4294967301</v>
       </c>
       <c r="AO7">
-        <v>4294967301</v>
+        <v>9999999.93999999947846</v>
       </c>
       <c r="AP7">
-        <v>4294967301</v>
+        <v>9999999.93999999947846</v>
       </c>
       <c r="AQ7">
         <v>9999999.93999999947846</v>
@@ -2648,10 +2609,10 @@
         <v>9999999.93999999947846</v>
       </c>
       <c r="AS7">
-        <v>9999999.93999999947846</v>
+        <v>99999999.93999999761581</v>
       </c>
       <c r="AT7">
-        <v>9999999.93999999947846</v>
+        <v>99999999.93999999761581</v>
       </c>
       <c r="AU7">
         <v>99999999.93999999761581</v>
@@ -2659,11 +2620,11 @@
       <c r="AV7">
         <v>99999999.93999999761581</v>
       </c>
-      <c r="AW7">
-        <v>99999999.93999999761581</v>
-      </c>
-      <c r="AX7">
-        <v>99999999.93999999761581</v>
+      <c r="AW7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="b">
+        <v>1</v>
       </c>
       <c r="AY7" t="b">
         <v>1</v>
@@ -2671,11 +2632,11 @@
       <c r="AZ7" t="b">
         <v>1</v>
       </c>
-      <c r="BA7" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB7" t="b">
-        <v>1</v>
+      <c r="BA7" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>158</v>
       </c>
       <c r="BC7" t="s">
         <v>159</v>
@@ -2711,75 +2672,69 @@
         <v>169</v>
       </c>
       <c r="BN7" t="s">
+        <v>169</v>
+      </c>
+      <c r="BO7" t="s">
+        <v>169</v>
+      </c>
+      <c r="BP7" t="s">
+        <v>169</v>
+      </c>
+      <c r="BQ7" t="s">
         <v>170</v>
       </c>
-      <c r="BO7" t="s">
+      <c r="BR7" t="s">
+        <v>170</v>
+      </c>
+      <c r="BS7" t="s">
+        <v>170</v>
+      </c>
+      <c r="BT7" t="s">
+        <v>170</v>
+      </c>
+      <c r="BU7" t="s">
         <v>171</v>
       </c>
-      <c r="BP7" t="s">
+      <c r="BV7" t="s">
         <v>171</v>
       </c>
-      <c r="BQ7" t="s">
+      <c r="BW7" t="s">
         <v>171</v>
       </c>
-      <c r="BR7" t="s">
+      <c r="BX7" t="s">
         <v>171</v>
       </c>
-      <c r="BS7" t="s">
+      <c r="BY7" t="s">
         <v>172</v>
       </c>
-      <c r="BT7" t="s">
+      <c r="BZ7" t="s">
         <v>172</v>
       </c>
-      <c r="BU7" t="s">
+      <c r="CA7" t="s">
         <v>172</v>
       </c>
-      <c r="BV7" t="s">
+      <c r="CB7" t="s">
         <v>172</v>
       </c>
-      <c r="BW7" t="s">
+      <c r="CC7" t="s">
         <v>173</v>
       </c>
-      <c r="BX7" t="s">
+      <c r="CD7" t="s">
         <v>173</v>
       </c>
-      <c r="BY7" t="s">
+      <c r="CE7" t="s">
         <v>173</v>
       </c>
-      <c r="BZ7" t="s">
+      <c r="CF7" t="s">
         <v>173</v>
       </c>
-      <c r="CA7" t="s">
-        <v>174</v>
-      </c>
-      <c r="CB7" t="s">
-        <v>174</v>
-      </c>
-      <c r="CC7" t="s">
-        <v>174</v>
-      </c>
-      <c r="CD7" t="s">
-        <v>174</v>
-      </c>
-      <c r="CE7" t="s">
-        <v>175</v>
-      </c>
-      <c r="CF7" t="s">
-        <v>175</v>
-      </c>
-      <c r="CG7" t="s">
-        <v>175</v>
-      </c>
-      <c r="CH7" t="s">
-        <v>175</v>
-      </c>
     </row>
-    <row r="8" spans="1:86">
+    <row r="8" spans="1:84">
       <c r="A8">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="C8">
         <v>121</v>
@@ -2788,10 +2743,10 @@
         <v>121</v>
       </c>
       <c r="E8">
-        <v>121</v>
+        <v>249</v>
       </c>
       <c r="F8">
-        <v>121</v>
+        <v>249</v>
       </c>
       <c r="G8">
         <v>249</v>
@@ -2800,10 +2755,10 @@
         <v>249</v>
       </c>
       <c r="I8">
-        <v>249</v>
+        <v>32761</v>
       </c>
       <c r="J8">
-        <v>249</v>
+        <v>32761</v>
       </c>
       <c r="K8">
         <v>32761</v>
@@ -2812,10 +2767,10 @@
         <v>32761</v>
       </c>
       <c r="M8">
-        <v>32761</v>
+        <v>65529</v>
       </c>
       <c r="N8">
-        <v>32761</v>
+        <v>65529</v>
       </c>
       <c r="O8">
         <v>65529</v>
@@ -2824,10 +2779,10 @@
         <v>65529</v>
       </c>
       <c r="Q8">
-        <v>65529</v>
+        <v>8388601</v>
       </c>
       <c r="R8">
-        <v>65529</v>
+        <v>8388601</v>
       </c>
       <c r="S8">
         <v>8388601</v>
@@ -2836,10 +2791,10 @@
         <v>8388601</v>
       </c>
       <c r="U8">
-        <v>8388601</v>
+        <v>16777209</v>
       </c>
       <c r="V8">
-        <v>8388601</v>
+        <v>16777209</v>
       </c>
       <c r="W8">
         <v>16777209</v>
@@ -2848,10 +2803,10 @@
         <v>16777209</v>
       </c>
       <c r="Y8">
-        <v>16777209</v>
+        <v>2147483641</v>
       </c>
       <c r="Z8">
-        <v>16777209</v>
+        <v>2147483641</v>
       </c>
       <c r="AA8">
         <v>2147483641</v>
@@ -2860,10 +2815,10 @@
         <v>2147483641</v>
       </c>
       <c r="AC8">
-        <v>2147483641</v>
+        <v>4294967289</v>
       </c>
       <c r="AD8">
-        <v>2147483641</v>
+        <v>4294967289</v>
       </c>
       <c r="AE8">
         <v>4294967289</v>
@@ -2872,22 +2827,22 @@
         <v>4294967289</v>
       </c>
       <c r="AG8">
-        <v>4294967289</v>
+        <v>2147483652</v>
       </c>
       <c r="AH8">
-        <v>4294967289</v>
+        <v>2147483651</v>
       </c>
       <c r="AI8">
         <v>2147483652</v>
       </c>
       <c r="AJ8">
-        <v>2147483651</v>
+        <v>2147483652</v>
       </c>
       <c r="AK8">
-        <v>2147483652</v>
+        <v>4294967300</v>
       </c>
       <c r="AL8">
-        <v>2147483652</v>
+        <v>4294967300</v>
       </c>
       <c r="AM8">
         <v>4294967300</v>
@@ -2896,10 +2851,10 @@
         <v>4294967300</v>
       </c>
       <c r="AO8">
-        <v>4294967300</v>
+        <v>9999999.92999999970198</v>
       </c>
       <c r="AP8">
-        <v>4294967300</v>
+        <v>9999999.92999999970198</v>
       </c>
       <c r="AQ8">
         <v>9999999.92999999970198</v>
@@ -2908,10 +2863,10 @@
         <v>9999999.92999999970198</v>
       </c>
       <c r="AS8">
-        <v>9999999.92999999970198</v>
+        <v>99999999.9299999922514</v>
       </c>
       <c r="AT8">
-        <v>9999999.92999999970198</v>
+        <v>99999999.9299999922514</v>
       </c>
       <c r="AU8">
         <v>99999999.9299999922514</v>
@@ -2919,11 +2874,11 @@
       <c r="AV8">
         <v>99999999.9299999922514</v>
       </c>
-      <c r="AW8">
-        <v>99999999.9299999922514</v>
-      </c>
-      <c r="AX8">
-        <v>99999999.9299999922514</v>
+      <c r="AW8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX8" t="b">
+        <v>1</v>
       </c>
       <c r="AY8" t="b">
         <v>1</v>
@@ -2931,11 +2886,11 @@
       <c r="AZ8" t="b">
         <v>1</v>
       </c>
-      <c r="BA8" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB8" t="b">
-        <v>1</v>
+      <c r="BA8" t="s">
+        <v>174</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>175</v>
       </c>
       <c r="BC8" t="s">
         <v>176</v>
@@ -2971,75 +2926,69 @@
         <v>186</v>
       </c>
       <c r="BN8" t="s">
+        <v>186</v>
+      </c>
+      <c r="BO8" t="s">
+        <v>186</v>
+      </c>
+      <c r="BP8" t="s">
+        <v>186</v>
+      </c>
+      <c r="BQ8" t="s">
         <v>187</v>
       </c>
-      <c r="BO8" t="s">
+      <c r="BR8" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS8" t="s">
+        <v>187</v>
+      </c>
+      <c r="BT8" t="s">
+        <v>187</v>
+      </c>
+      <c r="BU8" t="s">
         <v>188</v>
       </c>
-      <c r="BP8" t="s">
+      <c r="BV8" t="s">
         <v>188</v>
       </c>
-      <c r="BQ8" t="s">
+      <c r="BW8" t="s">
         <v>188</v>
       </c>
-      <c r="BR8" t="s">
+      <c r="BX8" t="s">
         <v>188</v>
       </c>
-      <c r="BS8" t="s">
+      <c r="BY8" t="s">
         <v>189</v>
       </c>
-      <c r="BT8" t="s">
+      <c r="BZ8" t="s">
         <v>189</v>
       </c>
-      <c r="BU8" t="s">
+      <c r="CA8" t="s">
         <v>189</v>
       </c>
-      <c r="BV8" t="s">
+      <c r="CB8" t="s">
         <v>189</v>
       </c>
-      <c r="BW8" t="s">
+      <c r="CC8" t="s">
         <v>190</v>
       </c>
-      <c r="BX8" t="s">
+      <c r="CD8" t="s">
         <v>190</v>
       </c>
-      <c r="BY8" t="s">
+      <c r="CE8" t="s">
         <v>190</v>
       </c>
-      <c r="BZ8" t="s">
+      <c r="CF8" t="s">
         <v>190</v>
       </c>
-      <c r="CA8" t="s">
-        <v>191</v>
-      </c>
-      <c r="CB8" t="s">
-        <v>191</v>
-      </c>
-      <c r="CC8" t="s">
-        <v>191</v>
-      </c>
-      <c r="CD8" t="s">
-        <v>191</v>
-      </c>
-      <c r="CE8" t="s">
-        <v>192</v>
-      </c>
-      <c r="CF8" t="s">
-        <v>192</v>
-      </c>
-      <c r="CG8" t="s">
-        <v>192</v>
-      </c>
-      <c r="CH8" t="s">
-        <v>192</v>
-      </c>
     </row>
-    <row r="9" spans="1:86">
+    <row r="9" spans="1:84">
       <c r="A9">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="C9">
         <v>120</v>
@@ -3048,10 +2997,10 @@
         <v>120</v>
       </c>
       <c r="E9">
-        <v>120</v>
+        <v>248</v>
       </c>
       <c r="F9">
-        <v>120</v>
+        <v>248</v>
       </c>
       <c r="G9">
         <v>248</v>
@@ -3060,10 +3009,10 @@
         <v>248</v>
       </c>
       <c r="I9">
-        <v>248</v>
+        <v>32760</v>
       </c>
       <c r="J9">
-        <v>248</v>
+        <v>32760</v>
       </c>
       <c r="K9">
         <v>32760</v>
@@ -3072,10 +3021,10 @@
         <v>32760</v>
       </c>
       <c r="M9">
-        <v>32760</v>
+        <v>65528</v>
       </c>
       <c r="N9">
-        <v>32760</v>
+        <v>65528</v>
       </c>
       <c r="O9">
         <v>65528</v>
@@ -3084,10 +3033,10 @@
         <v>65528</v>
       </c>
       <c r="Q9">
-        <v>65528</v>
+        <v>8388600</v>
       </c>
       <c r="R9">
-        <v>65528</v>
+        <v>8388600</v>
       </c>
       <c r="S9">
         <v>8388600</v>
@@ -3096,10 +3045,10 @@
         <v>8388600</v>
       </c>
       <c r="U9">
-        <v>8388600</v>
+        <v>16777208</v>
       </c>
       <c r="V9">
-        <v>8388600</v>
+        <v>16777208</v>
       </c>
       <c r="W9">
         <v>16777208</v>
@@ -3108,10 +3057,10 @@
         <v>16777208</v>
       </c>
       <c r="Y9">
-        <v>16777208</v>
+        <v>2147483640</v>
       </c>
       <c r="Z9">
-        <v>16777208</v>
+        <v>2147483640</v>
       </c>
       <c r="AA9">
         <v>2147483640</v>
@@ -3120,10 +3069,10 @@
         <v>2147483640</v>
       </c>
       <c r="AC9">
-        <v>2147483640</v>
+        <v>4294967288</v>
       </c>
       <c r="AD9">
-        <v>2147483640</v>
+        <v>4294967288</v>
       </c>
       <c r="AE9">
         <v>4294967288</v>
@@ -3132,10 +3081,10 @@
         <v>4294967288</v>
       </c>
       <c r="AG9">
-        <v>4294967288</v>
+        <v>2147483651</v>
       </c>
       <c r="AH9">
-        <v>4294967288</v>
+        <v>2147483651</v>
       </c>
       <c r="AI9">
         <v>2147483651</v>
@@ -3144,10 +3093,10 @@
         <v>2147483651</v>
       </c>
       <c r="AK9">
-        <v>2147483651</v>
+        <v>4294967299</v>
       </c>
       <c r="AL9">
-        <v>2147483651</v>
+        <v>4294967299</v>
       </c>
       <c r="AM9">
         <v>4294967299</v>
@@ -3156,10 +3105,10 @@
         <v>4294967299</v>
       </c>
       <c r="AO9">
-        <v>4294967299</v>
+        <v>9999999.91999999992549</v>
       </c>
       <c r="AP9">
-        <v>4294967299</v>
+        <v>9999999.91999999992549</v>
       </c>
       <c r="AQ9">
         <v>9999999.91999999992549</v>
@@ -3168,10 +3117,10 @@
         <v>9999999.91999999992549</v>
       </c>
       <c r="AS9">
-        <v>9999999.91999999992549</v>
+        <v>99999999.92000000178814</v>
       </c>
       <c r="AT9">
-        <v>9999999.91999999992549</v>
+        <v>99999999.92000000178814</v>
       </c>
       <c r="AU9">
         <v>99999999.92000000178814</v>
@@ -3179,11 +3128,11 @@
       <c r="AV9">
         <v>99999999.92000000178814</v>
       </c>
-      <c r="AW9">
-        <v>99999999.92000000178814</v>
-      </c>
-      <c r="AX9">
-        <v>99999999.92000000178814</v>
+      <c r="AW9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX9" t="b">
+        <v>1</v>
       </c>
       <c r="AY9" t="b">
         <v>1</v>
@@ -3191,11 +3140,11 @@
       <c r="AZ9" t="b">
         <v>1</v>
       </c>
-      <c r="BA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB9" t="b">
-        <v>1</v>
+      <c r="BA9" t="s">
+        <v>191</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>192</v>
       </c>
       <c r="BC9" t="s">
         <v>193</v>
@@ -3231,75 +3180,69 @@
         <v>203</v>
       </c>
       <c r="BN9" t="s">
+        <v>203</v>
+      </c>
+      <c r="BO9" t="s">
+        <v>203</v>
+      </c>
+      <c r="BP9" t="s">
+        <v>203</v>
+      </c>
+      <c r="BQ9" t="s">
         <v>204</v>
       </c>
-      <c r="BO9" t="s">
+      <c r="BR9" t="s">
+        <v>204</v>
+      </c>
+      <c r="BS9" t="s">
+        <v>204</v>
+      </c>
+      <c r="BT9" t="s">
+        <v>204</v>
+      </c>
+      <c r="BU9" t="s">
         <v>205</v>
       </c>
-      <c r="BP9" t="s">
+      <c r="BV9" t="s">
         <v>205</v>
       </c>
-      <c r="BQ9" t="s">
+      <c r="BW9" t="s">
         <v>205</v>
       </c>
-      <c r="BR9" t="s">
+      <c r="BX9" t="s">
         <v>205</v>
       </c>
-      <c r="BS9" t="s">
+      <c r="BY9" t="s">
         <v>206</v>
       </c>
-      <c r="BT9" t="s">
+      <c r="BZ9" t="s">
         <v>206</v>
       </c>
-      <c r="BU9" t="s">
+      <c r="CA9" t="s">
         <v>206</v>
       </c>
-      <c r="BV9" t="s">
+      <c r="CB9" t="s">
         <v>206</v>
       </c>
-      <c r="BW9" t="s">
+      <c r="CC9" t="s">
         <v>207</v>
       </c>
-      <c r="BX9" t="s">
+      <c r="CD9" t="s">
         <v>207</v>
       </c>
-      <c r="BY9" t="s">
+      <c r="CE9" t="s">
         <v>207</v>
       </c>
-      <c r="BZ9" t="s">
+      <c r="CF9" t="s">
         <v>207</v>
       </c>
-      <c r="CA9" t="s">
-        <v>208</v>
-      </c>
-      <c r="CB9" t="s">
-        <v>208</v>
-      </c>
-      <c r="CC9" t="s">
-        <v>208</v>
-      </c>
-      <c r="CD9" t="s">
-        <v>208</v>
-      </c>
-      <c r="CE9" t="s">
-        <v>209</v>
-      </c>
-      <c r="CF9" t="s">
-        <v>209</v>
-      </c>
-      <c r="CG9" t="s">
-        <v>209</v>
-      </c>
-      <c r="CH9" t="s">
-        <v>209</v>
-      </c>
     </row>
-    <row r="10" spans="1:86">
+    <row r="10" spans="1:84">
       <c r="A10">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="C10">
         <v>119</v>
@@ -3308,10 +3251,10 @@
         <v>119</v>
       </c>
       <c r="E10">
-        <v>119</v>
+        <v>247</v>
       </c>
       <c r="F10">
-        <v>119</v>
+        <v>247</v>
       </c>
       <c r="G10">
         <v>247</v>
@@ -3320,10 +3263,10 @@
         <v>247</v>
       </c>
       <c r="I10">
-        <v>247</v>
+        <v>32759</v>
       </c>
       <c r="J10">
-        <v>247</v>
+        <v>32759</v>
       </c>
       <c r="K10">
         <v>32759</v>
@@ -3332,10 +3275,10 @@
         <v>32759</v>
       </c>
       <c r="M10">
-        <v>32759</v>
+        <v>65527</v>
       </c>
       <c r="N10">
-        <v>32759</v>
+        <v>65527</v>
       </c>
       <c r="O10">
         <v>65527</v>
@@ -3344,10 +3287,10 @@
         <v>65527</v>
       </c>
       <c r="Q10">
-        <v>65527</v>
+        <v>8388599</v>
       </c>
       <c r="R10">
-        <v>65527</v>
+        <v>8388599</v>
       </c>
       <c r="S10">
         <v>8388599</v>
@@ -3356,10 +3299,10 @@
         <v>8388599</v>
       </c>
       <c r="U10">
-        <v>8388599</v>
+        <v>16777207</v>
       </c>
       <c r="V10">
-        <v>8388599</v>
+        <v>16777207</v>
       </c>
       <c r="W10">
         <v>16777207</v>
@@ -3368,10 +3311,10 @@
         <v>16777207</v>
       </c>
       <c r="Y10">
-        <v>16777207</v>
+        <v>2147483639</v>
       </c>
       <c r="Z10">
-        <v>16777207</v>
+        <v>2147483639</v>
       </c>
       <c r="AA10">
         <v>2147483639</v>
@@ -3380,10 +3323,10 @@
         <v>2147483639</v>
       </c>
       <c r="AC10">
-        <v>2147483639</v>
+        <v>4294967287</v>
       </c>
       <c r="AD10">
-        <v>2147483639</v>
+        <v>4294967287</v>
       </c>
       <c r="AE10">
         <v>4294967287</v>
@@ -3392,10 +3335,10 @@
         <v>4294967287</v>
       </c>
       <c r="AG10">
-        <v>4294967287</v>
+        <v>2147483650</v>
       </c>
       <c r="AH10">
-        <v>4294967287</v>
+        <v>2147483650</v>
       </c>
       <c r="AI10">
         <v>2147483650</v>
@@ -3404,10 +3347,10 @@
         <v>2147483650</v>
       </c>
       <c r="AK10">
-        <v>2147483650</v>
+        <v>4294967298</v>
       </c>
       <c r="AL10">
-        <v>2147483650</v>
+        <v>4294967298</v>
       </c>
       <c r="AM10">
         <v>4294967298</v>
@@ -3416,10 +3359,10 @@
         <v>4294967298</v>
       </c>
       <c r="AO10">
-        <v>4294967298</v>
+        <v>9999999.91000000014901</v>
       </c>
       <c r="AP10">
-        <v>4294967298</v>
+        <v>9999999.91000000014901</v>
       </c>
       <c r="AQ10">
         <v>9999999.91000000014901</v>
@@ -3428,10 +3371,10 @@
         <v>9999999.91000000014901</v>
       </c>
       <c r="AS10">
-        <v>9999999.91000000014901</v>
+        <v>99999999.90999999642372</v>
       </c>
       <c r="AT10">
-        <v>9999999.91000000014901</v>
+        <v>99999999.90999999642372</v>
       </c>
       <c r="AU10">
         <v>99999999.90999999642372</v>
@@ -3439,11 +3382,11 @@
       <c r="AV10">
         <v>99999999.90999999642372</v>
       </c>
-      <c r="AW10">
-        <v>99999999.90999999642372</v>
-      </c>
-      <c r="AX10">
-        <v>99999999.90999999642372</v>
+      <c r="AW10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX10" t="b">
+        <v>1</v>
       </c>
       <c r="AY10" t="b">
         <v>1</v>
@@ -3451,11 +3394,11 @@
       <c r="AZ10" t="b">
         <v>1</v>
       </c>
-      <c r="BA10" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB10" t="b">
-        <v>1</v>
+      <c r="BA10" t="s">
+        <v>208</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>209</v>
       </c>
       <c r="BC10" t="s">
         <v>210</v>
@@ -3491,75 +3434,69 @@
         <v>220</v>
       </c>
       <c r="BN10" t="s">
+        <v>220</v>
+      </c>
+      <c r="BO10" t="s">
+        <v>220</v>
+      </c>
+      <c r="BP10" t="s">
+        <v>220</v>
+      </c>
+      <c r="BQ10" t="s">
         <v>221</v>
       </c>
-      <c r="BO10" t="s">
+      <c r="BR10" t="s">
+        <v>221</v>
+      </c>
+      <c r="BS10" t="s">
+        <v>221</v>
+      </c>
+      <c r="BT10" t="s">
+        <v>221</v>
+      </c>
+      <c r="BU10" t="s">
         <v>222</v>
       </c>
-      <c r="BP10" t="s">
+      <c r="BV10" t="s">
         <v>222</v>
       </c>
-      <c r="BQ10" t="s">
+      <c r="BW10" t="s">
         <v>222</v>
       </c>
-      <c r="BR10" t="s">
+      <c r="BX10" t="s">
         <v>222</v>
       </c>
-      <c r="BS10" t="s">
+      <c r="BY10" t="s">
         <v>223</v>
       </c>
-      <c r="BT10" t="s">
+      <c r="BZ10" t="s">
         <v>223</v>
       </c>
-      <c r="BU10" t="s">
+      <c r="CA10" t="s">
         <v>223</v>
       </c>
-      <c r="BV10" t="s">
+      <c r="CB10" t="s">
         <v>223</v>
       </c>
-      <c r="BW10" t="s">
+      <c r="CC10" t="s">
         <v>224</v>
       </c>
-      <c r="BX10" t="s">
+      <c r="CD10" t="s">
         <v>224</v>
       </c>
-      <c r="BY10" t="s">
+      <c r="CE10" t="s">
         <v>224</v>
       </c>
-      <c r="BZ10" t="s">
+      <c r="CF10" t="s">
         <v>224</v>
       </c>
-      <c r="CA10" t="s">
-        <v>225</v>
-      </c>
-      <c r="CB10" t="s">
-        <v>225</v>
-      </c>
-      <c r="CC10" t="s">
-        <v>225</v>
-      </c>
-      <c r="CD10" t="s">
-        <v>225</v>
-      </c>
-      <c r="CE10" t="s">
-        <v>226</v>
-      </c>
-      <c r="CF10" t="s">
-        <v>226</v>
-      </c>
-      <c r="CG10" t="s">
-        <v>226</v>
-      </c>
-      <c r="CH10" t="s">
-        <v>226</v>
-      </c>
     </row>
-    <row r="11" spans="1:86">
+    <row r="11" spans="1:84">
       <c r="A11">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="C11">
         <v>118</v>
@@ -3568,10 +3505,10 @@
         <v>118</v>
       </c>
       <c r="E11">
-        <v>118</v>
+        <v>246</v>
       </c>
       <c r="F11">
-        <v>118</v>
+        <v>246</v>
       </c>
       <c r="G11">
         <v>246</v>
@@ -3580,10 +3517,10 @@
         <v>246</v>
       </c>
       <c r="I11">
-        <v>246</v>
+        <v>32758</v>
       </c>
       <c r="J11">
-        <v>246</v>
+        <v>32758</v>
       </c>
       <c r="K11">
         <v>32758</v>
@@ -3592,10 +3529,10 @@
         <v>32758</v>
       </c>
       <c r="M11">
-        <v>32758</v>
+        <v>65526</v>
       </c>
       <c r="N11">
-        <v>32758</v>
+        <v>65526</v>
       </c>
       <c r="O11">
         <v>65526</v>
@@ -3604,10 +3541,10 @@
         <v>65526</v>
       </c>
       <c r="Q11">
-        <v>65526</v>
+        <v>8388598</v>
       </c>
       <c r="R11">
-        <v>65526</v>
+        <v>8388598</v>
       </c>
       <c r="S11">
         <v>8388598</v>
@@ -3616,10 +3553,10 @@
         <v>8388598</v>
       </c>
       <c r="U11">
-        <v>8388598</v>
+        <v>16777206</v>
       </c>
       <c r="V11">
-        <v>8388598</v>
+        <v>16777206</v>
       </c>
       <c r="W11">
         <v>16777206</v>
@@ -3628,10 +3565,10 @@
         <v>16777206</v>
       </c>
       <c r="Y11">
-        <v>16777206</v>
+        <v>2147483638</v>
       </c>
       <c r="Z11">
-        <v>16777206</v>
+        <v>2147483638</v>
       </c>
       <c r="AA11">
         <v>2147483638</v>
@@ -3640,10 +3577,10 @@
         <v>2147483638</v>
       </c>
       <c r="AC11">
-        <v>2147483638</v>
+        <v>4294967286</v>
       </c>
       <c r="AD11">
-        <v>2147483638</v>
+        <v>4294967286</v>
       </c>
       <c r="AE11">
         <v>4294967286</v>
@@ -3652,10 +3589,10 @@
         <v>4294967286</v>
       </c>
       <c r="AG11">
-        <v>4294967286</v>
+        <v>2147483649</v>
       </c>
       <c r="AH11">
-        <v>4294967286</v>
+        <v>2147483649</v>
       </c>
       <c r="AI11">
         <v>2147483649</v>
@@ -3664,10 +3601,10 @@
         <v>2147483649</v>
       </c>
       <c r="AK11">
-        <v>2147483649</v>
+        <v>4294967297</v>
       </c>
       <c r="AL11">
-        <v>2147483649</v>
+        <v>4294967297</v>
       </c>
       <c r="AM11">
         <v>4294967297</v>
@@ -3676,10 +3613,10 @@
         <v>4294967297</v>
       </c>
       <c r="AO11">
-        <v>4294967297</v>
+        <v>9999999.90000000037253</v>
       </c>
       <c r="AP11">
-        <v>4294967297</v>
+        <v>9999999.90000000037253</v>
       </c>
       <c r="AQ11">
         <v>9999999.90000000037253</v>
@@ -3688,10 +3625,10 @@
         <v>9999999.90000000037253</v>
       </c>
       <c r="AS11">
-        <v>9999999.90000000037253</v>
+        <v>99999999.8999999910593</v>
       </c>
       <c r="AT11">
-        <v>9999999.90000000037253</v>
+        <v>99999999.8999999910593</v>
       </c>
       <c r="AU11">
         <v>99999999.8999999910593</v>
@@ -3699,11 +3636,11 @@
       <c r="AV11">
         <v>99999999.8999999910593</v>
       </c>
-      <c r="AW11">
-        <v>99999999.8999999910593</v>
-      </c>
-      <c r="AX11">
-        <v>99999999.8999999910593</v>
+      <c r="AW11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AX11" t="b">
+        <v>1</v>
       </c>
       <c r="AY11" t="b">
         <v>1</v>
@@ -3711,11 +3648,11 @@
       <c r="AZ11" t="b">
         <v>1</v>
       </c>
-      <c r="BA11" t="b">
-        <v>1</v>
-      </c>
-      <c r="BB11" t="b">
-        <v>1</v>
+      <c r="BA11" t="s">
+        <v>225</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>226</v>
       </c>
       <c r="BC11" t="s">
         <v>227</v>
@@ -3751,67 +3688,61 @@
         <v>237</v>
       </c>
       <c r="BN11" t="s">
+        <v>237</v>
+      </c>
+      <c r="BO11" t="s">
+        <v>237</v>
+      </c>
+      <c r="BP11" t="s">
+        <v>237</v>
+      </c>
+      <c r="BQ11" t="s">
         <v>238</v>
       </c>
-      <c r="BO11" t="s">
+      <c r="BR11" t="s">
+        <v>238</v>
+      </c>
+      <c r="BS11" t="s">
+        <v>238</v>
+      </c>
+      <c r="BT11" t="s">
+        <v>238</v>
+      </c>
+      <c r="BU11" t="s">
         <v>239</v>
       </c>
-      <c r="BP11" t="s">
+      <c r="BV11" t="s">
         <v>239</v>
       </c>
-      <c r="BQ11" t="s">
+      <c r="BW11" t="s">
         <v>239</v>
       </c>
-      <c r="BR11" t="s">
+      <c r="BX11" t="s">
         <v>239</v>
       </c>
-      <c r="BS11" t="s">
+      <c r="BY11" t="s">
         <v>240</v>
       </c>
-      <c r="BT11" t="s">
+      <c r="BZ11" t="s">
         <v>240</v>
       </c>
-      <c r="BU11" t="s">
+      <c r="CA11" t="s">
         <v>240</v>
       </c>
-      <c r="BV11" t="s">
+      <c r="CB11" t="s">
         <v>240</v>
       </c>
-      <c r="BW11" t="s">
+      <c r="CC11" t="s">
         <v>241</v>
       </c>
-      <c r="BX11" t="s">
+      <c r="CD11" t="s">
         <v>241</v>
       </c>
-      <c r="BY11" t="s">
+      <c r="CE11" t="s">
         <v>241</v>
       </c>
-      <c r="BZ11" t="s">
+      <c r="CF11" t="s">
         <v>241</v>
-      </c>
-      <c r="CA11" t="s">
-        <v>242</v>
-      </c>
-      <c r="CB11" t="s">
-        <v>242</v>
-      </c>
-      <c r="CC11" t="s">
-        <v>242</v>
-      </c>
-      <c r="CD11" t="s">
-        <v>242</v>
-      </c>
-      <c r="CE11" t="s">
-        <v>243</v>
-      </c>
-      <c r="CF11" t="s">
-        <v>243</v>
-      </c>
-      <c r="CG11" t="s">
-        <v>243</v>
-      </c>
-      <c r="CH11" t="s">
-        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>